<commit_message>
Add council speech scripts, raise meeting times, and tighten site chrome.
Ship the 3-minute speech picker and PDFs, put City Council meeting times under the TOC with live next dates, align on-page link order, remove action letter printables, and darken section borders so panels stay visible.
</commit_message>
<xml_diff>
--- a/docs/AI_Wrongful_Enforcement_Database.xlsx
+++ b/docs/AI_Wrongful_Enforcement_Database.xlsx
@@ -485,7 +485,7 @@
     <col width="18" customWidth="1" min="30" max="30"/>
     <col width="14" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="42" customWidth="1" min="33" max="33"/>
+    <col width="43" customWidth="1" min="33" max="33"/>
     <col width="17" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="15" customWidth="1" min="36" max="36"/>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="AZ3" s="3" t="inlineStr">
         <is>
-          <t>Vendor not confirmed in court opinion. Settlement authorized by SF Board of Supervisors Ordinance 181-15 ($495,000). Not a Flock Safety product case — cited as ALPR wrongful-stop liability scale only.</t>
+          <t>Vendor not confirmed in court opinion. Settlement authorized by SF Board of Supervisors Ordinance 181-15 ($495,000). Not a Flock Safety product case, cited as ALPR wrongful-stop liability scale only.</t>
         </is>
       </c>
       <c r="BA3" s="3" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Hofer and brother in a rental car stopped after ALPR flagged plate as stolen. Vehicle had previously been recovered; hot list not updated. High-risk stop with gun drawn; brother allegedly thrown to ground; car searched; ~40 minutes detention after rental app verification. Thanksgiving-period reporting conflict: Verge/filing (Nov 2018) vs EFF 'Thanksgiving 2019'—court/lawsuit timing supports late 2018.</t>
+          <t>Hofer and brother in a rental car stopped after ALPR flagged plate as stolen. Vehicle had previously been recovered; hot list not updated. High-risk stop with gun drawn; brother allegedly thrown to ground; car searched; ~40 minutes detention after rental app verification. Thanksgiving-period reporting conflict: Verge/filing (Nov 2018) vs EFF 'Thanksgiving 2019', court/lawsuit timing supports late 2018.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="AG4" s="2" t="inlineStr">
         <is>
-          <t>Partial—brother alleged injured</t>
+          <t>Partial, brother alleged injured</t>
         </is>
       </c>
       <c r="AH4" s="2" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="AZ8" s="2" t="inlineStr">
         <is>
-          <t>Vendor unspecified in major reporting. Spelling Brittney/Brittany varies in media; prefer Brittney (AP/CBS). Not a Flock Safety product case — cited as ALPR wrongful-stop liability scale only.</t>
+          <t>Vendor unspecified in major reporting. Spelling Brittney/Brittany varies in media; prefer Brittney (AP/CBS). Not a Flock Safety product case, cited as ALPR wrongful-stop liability scale only.</t>
         </is>
       </c>
       <c r="BA8" s="2" t="inlineStr">
@@ -3643,7 +3643,7 @@
       <c r="AF17" s="3" t="inlineStr"/>
       <c r="AG17" s="3" t="inlineStr">
         <is>
-          <t>Partial—contractions reported in custody</t>
+          <t>Partial, contractions reported in custody</t>
         </is>
       </c>
       <c r="AH17" s="3" t="inlineStr"/>
@@ -6389,7 +6389,7 @@
       </c>
       <c r="AM33" s="3" t="inlineStr">
         <is>
-          <t>~5.5 months (Jul 14–Dec 24, 2025)</t>
+          <t>~5.5 months (Jul 14-Dec 24, 2025)</t>
         </is>
       </c>
       <c r="AN33" s="3" t="inlineStr"/>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="AZ33" s="3" t="inlineStr">
         <is>
-          <t>Some reporting mentions Clearview AI / West Fargo role; primary Fargo investigation attribution varies — Vendor left NULL unless court docs confirm. Fox cited probation hold nuance; still FRT-linked extradition detention.</t>
+          <t>Some reporting mentions Clearview AI / West Fargo role; primary Fargo investigation attribution varies: Vendor left NULL unless court docs confirm. Fox cited probation hold nuance; still FRT-linked extradition detention.</t>
         </is>
       </c>
       <c r="BA33" s="3" t="inlineStr">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="Y43" s="3" t="inlineStr">
         <is>
-          <t>Partial—hands on guns</t>
+          <t>Partial, hands on guns</t>
         </is>
       </c>
       <c r="Z43" s="3" t="inlineStr"/>

</xml_diff>